<commit_message>
French to english comments, complementary datasets, 4/4 success
</commit_message>
<xml_diff>
--- a/data_target/results.xlsx
+++ b/data_target/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS4"/>
+  <dimension ref="A1:AW13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -580,65 +580,85 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>mod_freq_full</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>mod_freq_above_frc</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>mod_freq_below_frc</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>onset_count</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
           <t>P1_meanF0</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>P1_maxF0</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>P1_duration</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>P1_HNR</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>P1_jitter</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>P2_meanF0</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>P2_minF0</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>P2_duration</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>P2_HNR</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>P2_jitter</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>peak_time</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>peak_novelty</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>F0_range</t>
         </is>
@@ -647,7 +667,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GaBa</t>
+          <t>NiAn</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -656,92 +676,94 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.22933333333333</v>
+        <v>8.309333333333333</v>
       </c>
       <c r="D2" t="n">
         <v>1.482666666666667</v>
       </c>
       <c r="E2" t="n">
-        <v>11.712</v>
+        <v>9.792</v>
       </c>
       <c r="F2" t="n">
-        <v>104.5338684696497</v>
+        <v>104.4625771901023</v>
       </c>
       <c r="G2" t="n">
-        <v>33.98712251083354</v>
+        <v>1.833498624903414</v>
       </c>
       <c r="H2" t="n">
-        <v>50.21548382560187</v>
+        <v>102.670417003383</v>
       </c>
       <c r="I2" t="n">
-        <v>130.1497022755108</v>
+        <v>108.942522001075</v>
       </c>
       <c r="J2" t="n">
-        <v>79.93421844990894</v>
+        <v>6.272104997692054</v>
       </c>
       <c r="K2" t="n">
-        <v>0.007378445586221974</v>
+        <v>0.004157113026043648</v>
       </c>
       <c r="L2" t="n">
-        <v>7.011814043247355e-05</v>
+        <v>3.979794170060354e-05</v>
       </c>
       <c r="M2" t="n">
-        <v>0.003393431197416708</v>
+        <v>0.002267301525502125</v>
       </c>
       <c r="N2" t="n">
-        <v>0.003087042704528261</v>
+        <v>0.00234837063916828</v>
       </c>
       <c r="O2" t="n">
-        <v>0.01018029359225012</v>
+        <v>0.006801904576506375</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1347107048940786</v>
+        <v>0.06836542530485766</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.9774574911145395</v>
+        <v>0.5775933137992459</v>
       </c>
       <c r="R2" t="n">
-        <v>0.03210119397544992</v>
+        <v>0.02492748360212068</v>
       </c>
       <c r="S2" t="n">
-        <v>0.02498530461329468</v>
-      </c>
-      <c r="T2" t="inlineStr"/>
+        <v>0.03032223580030828</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0593230060686584</v>
+      </c>
       <c r="U2" t="n">
-        <v>0.09630358192634977</v>
+        <v>0.07478245080636205</v>
       </c>
       <c r="V2" t="n">
-        <v>1000.739619215815</v>
+        <v>903.0582256939173</v>
       </c>
       <c r="W2" t="n">
-        <v>1501.887696730821</v>
+        <v>1337.217287014922</v>
       </c>
       <c r="X2" t="n">
-        <v>2536.76025015554</v>
+        <v>2483.157297287015</v>
       </c>
       <c r="Y2" t="n">
-        <v>1000.574406529644</v>
+        <v>904.1735294850279</v>
       </c>
       <c r="Z2" t="n">
-        <v>1506.902573828688</v>
+        <v>1330.77492131822</v>
       </c>
       <c r="AA2" t="n">
-        <v>2510.263857885156</v>
+        <v>2507.206788267492</v>
       </c>
       <c r="AB2" t="n">
-        <v>14.07045218523798</v>
+        <v>13.54909092843113</v>
       </c>
       <c r="AC2" t="n">
-        <v>16.25249705562657</v>
+        <v>14.85310253337641</v>
       </c>
       <c r="AD2" t="n">
-        <v>36.97479665715031</v>
+        <v>37.86773918734608</v>
       </c>
       <c r="AE2" t="n">
-        <v>-10.3982572284893</v>
+        <v>-4.946281425040515</v>
       </c>
       <c r="AF2" t="n">
-        <v>10.22933333333333</v>
+        <v>8.309333333333333</v>
       </c>
       <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr"/>
@@ -756,246 +778,190 @@
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GaBa</t>
+          <t>NiAn</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>glide</t>
+          <t>trill_r</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.75733333333334</v>
+        <v>17.0773125</v>
       </c>
       <c r="D3" t="n">
-        <v>1.504</v>
+        <v>1.482666666666667</v>
       </c>
       <c r="E3" t="n">
-        <v>22.26133333333333</v>
-      </c>
-      <c r="F3" t="n">
-        <v>102.2167149596238</v>
-      </c>
-      <c r="G3" t="n">
-        <v>33.89448927471447</v>
-      </c>
-      <c r="H3" t="n">
-        <v>47.00062241256325</v>
-      </c>
-      <c r="I3" t="n">
-        <v>139.6395331471671</v>
-      </c>
-      <c r="J3" t="n">
-        <v>92.63891073460383</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.01261183195394132</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.0001213841664355234</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.005150605897821327</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.003918260015002748</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.01545181769346398</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.06296592782571975</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.5314942073070333</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.02964313733574229</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0.0329114290653207</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.05234930142668357</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.08892941200722687</v>
-      </c>
-      <c r="V3" t="n">
-        <v>935.2562980817434</v>
-      </c>
-      <c r="W3" t="n">
-        <v>1550.109826887814</v>
-      </c>
-      <c r="X3" t="n">
-        <v>2873.25954716301</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>871.4099692553292</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1428.30845392638</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>3049.212999181547</v>
-      </c>
+        <v>18.56</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="n">
-        <v>6.790258741385572</v>
+        <v>18.35513854872234</v>
       </c>
       <c r="AC3" t="n">
-        <v>17.37030063716979</v>
+        <v>16.27594359178523</v>
       </c>
       <c r="AD3" t="n">
-        <v>33.81460531405944</v>
+        <v>34.65622284350136</v>
       </c>
       <c r="AE3" t="n">
-        <v>-11.61520749508289</v>
+        <v>-6.368819103020104</v>
       </c>
       <c r="AF3" t="n">
-        <v>20.75733333333333</v>
+        <v>17.0773125</v>
       </c>
       <c r="AG3" t="n">
-        <v>103.2191779035709</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>139.6612496678476</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>5.12</v>
-      </c>
+        <v>27.2290755777639</v>
+      </c>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="n">
-        <v>7.011896015984719</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>0.009428233745263741</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>51.70094273994953</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>51.70094273994953</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>15.63733333333333</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>1.17942151252772</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="n">
-        <v>5.12</v>
-      </c>
-      <c r="AR3" t="n">
-        <v>0.4229398888853222</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>-51.51823516362136</v>
-      </c>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LuBa</t>
+          <t>NiAn</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>vowel_a</t>
+          <t>glide</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>9.290666666666667</v>
+        <v>6.837333333333333</v>
       </c>
       <c r="D4" t="n">
-        <v>1.482666666666667</v>
+        <v>1.504</v>
       </c>
       <c r="E4" t="n">
-        <v>10.77333333333333</v>
+        <v>8.341333333333333</v>
       </c>
       <c r="F4" t="n">
-        <v>169.3623564924953</v>
+        <v>167.3213884167252</v>
       </c>
       <c r="G4" t="n">
-        <v>2.377878805887182</v>
+        <v>79.82404043706676</v>
       </c>
       <c r="H4" t="n">
-        <v>163.2146480227671</v>
+        <v>85.77935935449786</v>
       </c>
       <c r="I4" t="n">
-        <v>173.3177133770812</v>
+        <v>388.2233416419645</v>
       </c>
       <c r="J4" t="n">
-        <v>10.10306535431414</v>
+        <v>302.4439822874667</v>
       </c>
       <c r="K4" t="n">
-        <v>0.008072307303532335</v>
+        <v>0.006902776272764932</v>
       </c>
       <c r="L4" t="n">
-        <v>4.769190802581817e-05</v>
+        <v>4.13680800318293e-05</v>
       </c>
       <c r="M4" t="n">
-        <v>0.005007294877585342</v>
+        <v>0.003437206479182518</v>
       </c>
       <c r="N4" t="n">
-        <v>0.004349434832705242</v>
+        <v>0.003386298953797161</v>
       </c>
       <c r="O4" t="n">
-        <v>0.01502188463275603</v>
+        <v>0.01031161943754755</v>
       </c>
       <c r="P4" t="n">
-        <v>0.04882300262450871</v>
+        <v>0.06101093593466034</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.4573537911180756</v>
+        <v>0.5392566262677113</v>
       </c>
       <c r="R4" t="n">
-        <v>0.01176302574230913</v>
+        <v>0.03179302258821632</v>
       </c>
       <c r="S4" t="n">
-        <v>0.01638581914191158</v>
+        <v>0.0397958157638722</v>
       </c>
       <c r="T4" t="n">
-        <v>0.04111153652569779</v>
+        <v>0.05192664925686601</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0352890772269274</v>
+        <v>0.09537906776464897</v>
       </c>
       <c r="V4" t="n">
-        <v>867.4537780369182</v>
+        <v>767.3190111894434</v>
       </c>
       <c r="W4" t="n">
-        <v>1421.007890471918</v>
+        <v>1385.239150710124</v>
       </c>
       <c r="X4" t="n">
-        <v>2693.254347134618</v>
+        <v>2670.917719166066</v>
       </c>
       <c r="Y4" t="n">
-        <v>874.5451909412302</v>
+        <v>766.7900037566988</v>
       </c>
       <c r="Z4" t="n">
-        <v>1404.715135852536</v>
+        <v>1376.103221720093</v>
       </c>
       <c r="AA4" t="n">
-        <v>2678.084407677334</v>
+        <v>2652.8929106699</v>
       </c>
       <c r="AB4" t="n">
-        <v>15.84275152446181</v>
+        <v>7.016876603641203</v>
       </c>
       <c r="AC4" t="n">
-        <v>14.89584064215333</v>
+        <v>17.17246187880812</v>
       </c>
       <c r="AD4" t="n">
-        <v>37.43354871701171</v>
+        <v>38.74517373529617</v>
       </c>
       <c r="AE4" t="n">
-        <v>-5.084624447711332</v>
+        <v>-10.15597090368706</v>
       </c>
       <c r="AF4" t="n">
-        <v>9.290666666666667</v>
+        <v>6.837333333333333</v>
       </c>
       <c r="AG4" t="inlineStr"/>
       <c r="AH4" t="inlineStr"/>
@@ -1003,13 +969,1038 @@
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
+      <c r="AM4" t="n">
+        <v>1.024</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>31.43678742579851</v>
+      </c>
       <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
+      <c r="AP4" t="n">
+        <v>152.1835768081592</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>85.50775437100125</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>5.813333333333333</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>11.07699855350605</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>0.006379489913751584</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>1.024</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>3.541353973737699</v>
+      </c>
+      <c r="AW4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GaBa</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>vowel_a</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10.22933333333333</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.482666666666667</v>
+      </c>
+      <c r="E5" t="n">
+        <v>11.712</v>
+      </c>
+      <c r="F5" t="n">
+        <v>104.5338684696497</v>
+      </c>
+      <c r="G5" t="n">
+        <v>33.98712251083354</v>
+      </c>
+      <c r="H5" t="n">
+        <v>50.21548382560187</v>
+      </c>
+      <c r="I5" t="n">
+        <v>130.1497022755108</v>
+      </c>
+      <c r="J5" t="n">
+        <v>79.93421844990894</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.007378445586221974</v>
+      </c>
+      <c r="L5" t="n">
+        <v>7.011814043247355e-05</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.003393431197416708</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.003087042704528261</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.01018029359225012</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.1347107048940786</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.9774574911145395</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.03210119397544992</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.02498530461329468</v>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="n">
+        <v>0.09630358192634977</v>
+      </c>
+      <c r="V5" t="n">
+        <v>1000.739619215815</v>
+      </c>
+      <c r="W5" t="n">
+        <v>1501.887696730821</v>
+      </c>
+      <c r="X5" t="n">
+        <v>2536.76025015554</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>1000.574406529644</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>1506.902573828688</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>2510.263857885156</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>14.07045218523798</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>16.25249705562657</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>36.97479665715031</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>-10.3982572284893</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>10.22933333333333</v>
+      </c>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GaBa</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>trill_r</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>6.432</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.482666666666667</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7.914666666666666</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="n">
+        <v>14.68451899704757</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>15.54183144586114</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>38.91801459107392</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>-8.867967099465925</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>6.432</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>31.85868213841691</v>
+      </c>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GaBa</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>glide</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>20.75733333333334</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.504</v>
+      </c>
+      <c r="E7" t="n">
+        <v>22.26133333333333</v>
+      </c>
+      <c r="F7" t="n">
+        <v>102.2167149596238</v>
+      </c>
+      <c r="G7" t="n">
+        <v>33.89448927471447</v>
+      </c>
+      <c r="H7" t="n">
+        <v>47.00062241256325</v>
+      </c>
+      <c r="I7" t="n">
+        <v>139.6395331471671</v>
+      </c>
+      <c r="J7" t="n">
+        <v>92.63891073460383</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.01261183195394132</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.0001213841664355234</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.005150605897821327</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.003918260015002748</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.01545181769346398</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.06296592782571975</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.5314942073070333</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.02964313733574229</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.0329114290653207</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.05234930142668357</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0.08892941200722687</v>
+      </c>
+      <c r="V7" t="n">
+        <v>935.2562980817434</v>
+      </c>
+      <c r="W7" t="n">
+        <v>1550.109826887814</v>
+      </c>
+      <c r="X7" t="n">
+        <v>2873.25954716301</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>871.4099692553292</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>1428.30845392638</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>3049.212999181547</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>6.790258741385572</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>17.37030063716979</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>33.81460531405944</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>-11.61520749508289</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>20.75733333333333</v>
+      </c>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="n">
+        <v>103.2191779035709</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>139.6612496678476</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>7.011896015984719</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>0.009428233745263741</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>51.70094273994953</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>51.70094273994953</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>15.63733333333333</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>1.17942151252772</v>
+      </c>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0.4229398888853222</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>-51.51823516362136</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LuBa</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>vowel_a</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>9.290666666666667</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.482666666666667</v>
+      </c>
+      <c r="E8" t="n">
+        <v>10.77333333333333</v>
+      </c>
+      <c r="F8" t="n">
+        <v>169.3623564924953</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.377878805887182</v>
+      </c>
+      <c r="H8" t="n">
+        <v>163.2146480227671</v>
+      </c>
+      <c r="I8" t="n">
+        <v>173.3177133770812</v>
+      </c>
+      <c r="J8" t="n">
+        <v>10.10306535431414</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.008072307303532335</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4.769190802581817e-05</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.005007294877585342</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.004349434832705242</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.01502188463275603</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.04882300262450871</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.4573537911180756</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.01176302574230913</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.01638581914191158</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.04111153652569779</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.0352890772269274</v>
+      </c>
+      <c r="V8" t="n">
+        <v>867.4537780369182</v>
+      </c>
+      <c r="W8" t="n">
+        <v>1421.007890471918</v>
+      </c>
+      <c r="X8" t="n">
+        <v>2693.254347134618</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>874.5451909412302</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>1404.715135852536</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>2678.084407677334</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>15.84275152446181</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>14.89584064215333</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>37.43354871701171</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>-5.084624447711332</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>9.290666666666667</v>
+      </c>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LuBa</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>trill_r</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>13.81333333333333</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.482666666666667</v>
+      </c>
+      <c r="E9" t="n">
+        <v>15.296</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="n">
+        <v>13.4824501171275</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>16.17437512166667</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>35.56401425232905</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>-7.610160724358993</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>13.81333333333333</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>31.19571511291257</v>
+      </c>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="n">
+        <v>12</v>
+      </c>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LuBa</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>glide</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>6.314666666666667</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.504</v>
+      </c>
+      <c r="E10" t="n">
+        <v>7.818666666666667</v>
+      </c>
+      <c r="F10" t="n">
+        <v>217.9430735653357</v>
+      </c>
+      <c r="G10" t="n">
+        <v>28.42198543393842</v>
+      </c>
+      <c r="H10" t="n">
+        <v>149.9551620563849</v>
+      </c>
+      <c r="I10" t="n">
+        <v>242.8597847769712</v>
+      </c>
+      <c r="J10" t="n">
+        <v>92.90462272058636</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.002602089017217253</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1.194945436684424e-05</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.001299159218717663</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.001496938336009565</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.003897477656152988</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.01915049083289768</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.2144451697793937</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.007973003991959994</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.01108192910608527</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.01719727598438148</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.02391901197587998</v>
+      </c>
+      <c r="V10" t="n">
+        <v>935.3495275186035</v>
+      </c>
+      <c r="W10" t="n">
+        <v>1482.610984525949</v>
+      </c>
+      <c r="X10" t="n">
+        <v>2865.525450228438</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>956.8992376866403</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>1495.574896506629</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>2868.624224521276</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>20.66809045943156</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>19.53944217649021</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>39.16152464580372</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>-20.53240444052781</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>6.314666666666667</v>
+      </c>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="n">
+        <v>1.024</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>23.55000466677673</v>
+      </c>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="n">
+        <v>217.6980090580782</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>149.7939795448653</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>5.290666666666667</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>19.57577237669599</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0.002801721707518872</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>1.024</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>4.064969742193191</v>
+      </c>
+      <c r="AW10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AnMa</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>vowel_a</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>7.936</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.472</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9.407999999999999</v>
+      </c>
+      <c r="F11" t="n">
+        <v>90.19469974203163</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.4935721776343399</v>
+      </c>
+      <c r="H11" t="n">
+        <v>89.65876146396073</v>
+      </c>
+      <c r="I11" t="n">
+        <v>90.66923901246166</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1.01047754850093</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.009277886004442607</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.0001027273299759971</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.003540602027483704</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="n">
+        <v>0.01062180608245111</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.2440351417936122</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>2.200451940758098</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.1410967698152549</v>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="n">
+        <v>0.4232903094457647</v>
+      </c>
+      <c r="V11" t="n">
+        <v>837.8378450127418</v>
+      </c>
+      <c r="W11" t="n">
+        <v>1460.508780310143</v>
+      </c>
+      <c r="X11" t="n">
+        <v>2268.779746832474</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>837.3832977982639</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>1461.548139942351</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>2256.319705992133</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>10.57620072230345</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>9.934735638583092</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>38.03959374616798</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>11.0873106909951</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>7.936</v>
+      </c>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AnMa</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>trill_r</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>45.71733333333334</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="E12" t="n">
+        <v>47.02933333333333</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="n">
+        <v>10.98440332546702</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>15.0494467526486</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>30.56655976820665</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>12.66848684878745</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>45.71733333333334</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>16.14173228346457</v>
+      </c>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="n">
+        <v>13</v>
+      </c>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AnMa</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>glide</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>23.968</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="E13" t="n">
+        <v>24</v>
+      </c>
+      <c r="F13" t="n">
+        <v>288.2056133902657</v>
+      </c>
+      <c r="G13" t="n">
+        <v>52.45036246665978</v>
+      </c>
+      <c r="H13" t="n">
+        <v>152.693505348654</v>
+      </c>
+      <c r="I13" t="n">
+        <v>331.6024509088924</v>
+      </c>
+      <c r="J13" t="n">
+        <v>178.9089455602383</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.004192803349350329</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1.456147712754105e-05</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.002353985870160548</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.002353038317929045</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.007061957610481644</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.06360151515531072</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.5976984513597836</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.03543719437321927</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0.03995067200073634</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.04518449996328593</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.1063115831196578</v>
+      </c>
+      <c r="V13" t="n">
+        <v>921.8877754199852</v>
+      </c>
+      <c r="W13" t="n">
+        <v>1567.512697626214</v>
+      </c>
+      <c r="X13" t="n">
+        <v>2510.328063059447</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>932.759024868849</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>1533.152614684847</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>2519.623332319181</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>14.23116857741078</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>16.83108292689746</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>33.37475994044195</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>-0.2019258934756265</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>23.968</v>
+      </c>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="n">
+        <v>2.730666666666667</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>9.278040519313629</v>
+      </c>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="n">
+        <v>271.2975896133867</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>138.9499843741667</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>21.23733333333333</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>13.87915117310336</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>0.004634902878333394</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>2.730666666666667</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>1.106291458074674</v>
+      </c>
+      <c r="AW13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1022,7 +2013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1045,54 +2036,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GaBa</t>
+          <t>NiAn</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erreur sur tâche trill: Argument "Minimum pitch" has the value "undefined".
-</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LuBa</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Erreur sur tâche trill: Argument "Minimum pitch" has the value "undefined".
-</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>LuBa</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Erreur sur tâche glide: Argument "Minimum pitch" has the value "undefined".
-</t>
+          <t>Sync signal not found, skipping synchronization</t>
         </is>
       </c>
     </row>

</xml_diff>